<commit_message>
docs(git): follow Report 2 branching (develop, feature/*) and commit format
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/plan/CrabShare_Ke_hoach_code_21_ngay.xlsx
+++ b/docs/plan/CrabShare_Ke_hoach_code_21_ngay.xlsx
@@ -468,7 +468,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cả 4 máy chạy được API + web + mobile, đăng nhập tài khoản demo; Jira có đủ task; main được bảo vệ (PR + CI).</t>
+          <t xml:space="preserve">Cả 4 máy chạy được API + web + mobile, đăng nhập tài khoản demo; Jira có đủ task; main và develop được bảo vệ (PR + CI).</t>
         </is>
       </c>
     </row>
@@ -519,7 +519,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tiền về bằng webhook, chốt vốn, ký hợp đồng, nhật ký + sự kiện hộp + timeline, bằng chứng + thẩm định, giỏ hàng → đơn → đóng gói → hoàn tất, danh mục NĐT. Chiều D14 cả nhóm tích hợp trên main.</t>
+          <t xml:space="preserve">Tiền về bằng webhook, chốt vốn, ký hợp đồng, nhật ký + sự kiện hộp + timeline, bằng chứng + thẩm định, giỏ hàng → đơn → đóng gói → hoàn tất, danh mục NĐT. Chiều D14 cả nhóm tích hợp trên develop rồi gộp vào main.</t>
         </is>
       </c>
     </row>
@@ -632,38 +632,38 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Một task chỉ "Xong" khi: code + test của phần đó đã merge vào main qua PR có người duyệt, CI xanh, đã tự thử trên máy và thỏa cột "Hoàn thành khi".</t>
+          <t xml:space="preserve">Một task chỉ "Xong" khi: code + test của phần đó đã merge vào develop qua PR có người duyệt, CI xanh, đã tự thử trên máy và thỏa cột "Hoàn thành khi".</t>
         </is>
       </c>
     </row>
     <row r="27" ht="32" customHeight="1">
       <c r="A27" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">Git</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nhánh feature/&lt;Jira key&gt;-&lt;slug&gt; tạo từ develop, PR vào develop; commit dạng feat(scope): mô tả tiếng Anh (Report 2 mục 6.2). main chỉ nhận develop ở mỗi mốc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="32" customHeight="1">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">Trễ hạn</t>
         </is>
       </c>
-      <c r="B27" s="2" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Thấy sắp trễ thì báo ngay trong ngày, không đợi tới hạn. Trưởng nhóm điều chỉnh hoặc cắt phạm vi theo thứ tự đã thống nhất với thầy.</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="13" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">Nguyên tắc chung</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="30" customHeight="1">
-      <c r="A30" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">•</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tiền là số nguyên đồng. Không hiển thị lợi suất kỳ vọng ở bất kỳ màn hình / API nào (TL-05 §8, BR-49).</t>
         </is>
       </c>
     </row>
@@ -675,7 +675,7 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mỗi module đọc README trong backend/src/CrabShare.Api/Features/&lt;Module&gt;/ trước khi làm (use case, bảng, endpoint dự kiến, quy tắc).</t>
+          <t xml:space="preserve">Tiền là số nguyên đồng. Không hiển thị lợi suất kỳ vọng ở bất kỳ màn hình / API nào (TL-05 §8, BR-49).</t>
         </is>
       </c>
     </row>
@@ -687,7 +687,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đổi CSDL bằng migration mới V003, V004… — không sửa file cũ; sinh lại entity bằng backend/scripts/scaffold-db.ps1.</t>
+          <t xml:space="preserve">Mỗi module đọc README trong backend/src/CrabShare.Api/Features/&lt;Module&gt;/ trước khi làm (use case, bảng, endpoint dự kiến, quy tắc).</t>
         </is>
       </c>
     </row>
@@ -699,12 +699,24 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">Đổi CSDL bằng migration mới V003, V004… — không sửa file cũ; sinh lại entity bằng backend/scripts/scaffold-db.ps1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="30" customHeight="1">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">•</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">Mobile: đổi dữ liệu mẫu sang API bằng cách viết Api…Repository và đổi một dòng provider; thêm màn mới thì thêm vào test/pages_smoke_test.dart.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="19">
+  <mergeCells count="20">
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="C12:E12"/>
     <mergeCell ref="C13:E13"/>
@@ -720,10 +732,11 @@
     <mergeCell ref="B25:E25"/>
     <mergeCell ref="B26:E26"/>
     <mergeCell ref="B27:E27"/>
-    <mergeCell ref="B30:E30"/>
+    <mergeCell ref="B28:E28"/>
     <mergeCell ref="B31:E31"/>
     <mergeCell ref="B32:E32"/>
     <mergeCell ref="B33:E33"/>
+    <mergeCell ref="B34:E34"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" paperSize="9" fitToWidth="1" fitToHeight="0"/>
@@ -875,7 +888,7 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Khởi động: cả nhóm chạy được dự án, bảo vệ nhánh main, dựng board Jira</t>
+          <t xml:space="preserve">Khởi động: cả nhóm chạy được dự án, bảo vệ nhánh main/develop, dựng board Jira</t>
         </is>
       </c>
       <c r="F2" s="4">
@@ -889,7 +902,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mời 3 bạn vào repo GitHub; bật Branch protection cho main (bắt buộc PR, 1 người duyệt, CI xanh). Kiểm tra CI chạy xanh trên PR đầu tiên.</t>
+          <t xml:space="preserve">Mời 3 bạn vào repo GitHub; đặt develop làm nhánh mặc định; bật Branch protection cho main và develop (bắt buộc PR, 1 người duyệt, CI xanh). Kiểm tra CI chạy xanh trên PR đầu tiên.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -909,7 +922,7 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 máy chạy được API + web + mobile và đăng nhập demo; không ai push thẳng được lên main; Jira có đủ task, mỗi người kéo task D1 sang In Progress.</t>
+          <t xml:space="preserve">4 máy chạy được API + web + mobile và đăng nhập demo; không ai push thẳng được lên main/develop; Jira có đủ task, mỗi người kéo task D1 sang In Progress.</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -4835,7 +4848,7 @@
       </c>
       <c r="M48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Thêm bậc phí có hiệu lực từ ngày chọn; lô duyệt sau ngày đó dùng phí mới. Chiều: merge PR tồn, chạy demo M2 trên main.</t>
+          <t xml:space="preserve">Thêm bậc phí có hiệu lực từ ngày chọn; lô duyệt sau ngày đó dùng phí mới. Chiều: merge PR tồn vào develop, chạy demo M2, gộp develop → main.</t>
         </is>
       </c>
       <c r="N48" s="2" t="inlineStr">
@@ -7116,7 +7129,7 @@
       </c>
       <c r="I75" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đóng băng main, gắn tag v1.0, ghi release notes; tập dượt demo 2 lần, bấm giờ.</t>
+          <t xml:space="preserve">Gộp develop → main lần cuối, đóng băng main, gắn tag v1.0, ghi release notes; tập dượt demo 2 lần, bấm giờ.</t>
         </is>
       </c>
       <c r="J75" s="2" t="inlineStr">
@@ -7263,7 +7276,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TH-01 Khởi động: cả nhóm chạy được dự án, bảo vệ nhánh main, dựng board Jira
+          <t xml:space="preserve">TH-01 Khởi động: cả nhóm chạy được dự án, bảo vệ nhánh main/develop, dựng board Jira
 TH-02 Nhật ký kiểm toán dùng chung + khung job nền (ngày 1/2)</t>
         </is>
       </c>
@@ -8407,7 +8420,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Khởi động: cả nhóm chạy được dự án, bảo vệ nhánh main, dựng board Jira</t>
+          <t xml:space="preserve">Khởi động: cả nhóm chạy được dự án, bảo vệ nhánh main/develop, dựng board Jira</t>
         </is>
       </c>
       <c r="C5" s="15" t="inlineStr">

</xml_diff>

<commit_message>
docs(plan): add Jira keys, branch names and board link
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/plan/CrabShare_Ke_hoach_code_21_ngay.xlsx
+++ b/docs/plan/CrabShare_Ke_hoach_code_21_ngay.xlsx
@@ -620,7 +620,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nếu dùng Jira: import file CrabShare_Jira_import.csv; sau khi import điền mã CS-xx vào cột "Jira key". Tên nhánh git = feature/&lt;Jira key&gt;-&lt;slug&gt; (cột "Nhánh git").</t>
+          <t xml:space="preserve">Đã tạo trên Jira: 19 epic (CS-1 → CS-19), 74 task (CS-20 → CS-93), 3 sprint theo tuần. Trạng thái thật cập nhật trên Jira: https://nguyendaothien2003.atlassian.net/jira/software/projects/CS/boards/2/backlog. Cột "Nhánh git" là tên nhánh đúng của từng task.</t>
         </is>
       </c>
     </row>
@@ -763,7 +763,7 @@
     <col min="14" max="14" width="18" customWidth="1"/>
     <col min="15" max="15" width="9" customWidth="1"/>
     <col min="16" max="16" width="12" customWidth="1"/>
-    <col min="17" max="17" width="24" customWidth="1"/>
+    <col min="17" max="17" width="34" customWidth="1"/>
     <col min="18" max="18" width="10" customWidth="1"/>
     <col min="19" max="19" width="34" customWidth="1"/>
   </cols>
@@ -851,7 +851,7 @@
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nhánh git (slug)</t>
+          <t xml:space="preserve">Nhánh git</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
@@ -942,10 +942,14 @@
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">khoi-dong</t>
-        </is>
-      </c>
-      <c r="R2" s="2"/>
+          <t xml:space="preserve">feature/CS-20-khoi-dong</t>
+        </is>
+      </c>
+      <c r="R2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-20</t>
+        </is>
+      </c>
       <c r="S2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Họp 15 phút đầu ngày mỗi ngày (daily) trên nhóm chat.</t>
@@ -1029,10 +1033,14 @@
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">audit-log-job-nen</t>
-        </is>
-      </c>
-      <c r="R3" s="2"/>
+          <t xml:space="preserve">feature/CS-21-audit-log-job-nen</t>
+        </is>
+      </c>
+      <c r="R3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-21</t>
+        </is>
+      </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Mọi API đổi tiền / hợp đồng / chi phí chuẩn / trạng thái lô / quyết toán đều phải gọi IAuditLog.</t>
@@ -1116,10 +1124,14 @@
       </c>
       <c r="Q4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">dang-ky-ho-nuoi</t>
-        </is>
-      </c>
-      <c r="R4" s="2"/>
+          <t xml:space="preserve">feature/CS-22-dang-ky-ho-nuoi</t>
+        </is>
+      </c>
+      <c r="R4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-22</t>
+        </is>
+      </c>
       <c r="S4" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Copy cách viết Features/Auth.</t>
@@ -1203,10 +1215,14 @@
       </c>
       <c r="Q5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">tsk13-du-lieu</t>
-        </is>
-      </c>
-      <c r="R5" s="2"/>
+          <t xml:space="preserve">feature/CS-23-tsk13-du-lieu</t>
+        </is>
+      </c>
+      <c r="R5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-23</t>
+        </is>
+      </c>
       <c r="S5" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Ảnh không commit vào git — để trên Drive nhóm.</t>
@@ -1290,10 +1306,14 @@
       </c>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">mobile-android</t>
-        </is>
-      </c>
-      <c r="R6" s="2"/>
+          <t xml:space="preserve">feature/CS-24-mobile-android</t>
+        </is>
+      </c>
+      <c r="R6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-24</t>
+        </is>
+      </c>
       <c r="S6" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Hướng dẫn cả nhóm chạy mobile.</t>
@@ -1377,10 +1397,14 @@
       </c>
       <c r="Q7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">duyet-ho-nuoi</t>
-        </is>
-      </c>
-      <c r="R7" s="2"/>
+          <t xml:space="preserve">feature/CS-25-duyet-ho-nuoi</t>
+        </is>
+      </c>
+      <c r="R7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-25</t>
+        </is>
+      </c>
       <c r="S7" s="2"/>
     </row>
     <row r="8">
@@ -1460,10 +1484,14 @@
       </c>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">niem-yet</t>
-        </is>
-      </c>
-      <c r="R8" s="2"/>
+          <t xml:space="preserve">feature/CS-26-niem-yet</t>
+        </is>
+      </c>
+      <c r="R8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-26</t>
+        </is>
+      </c>
       <c r="S8" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">TL-27.</t>
@@ -1547,10 +1575,14 @@
       </c>
       <c r="Q9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ekyc</t>
-        </is>
-      </c>
-      <c r="R9" s="2"/>
+          <t xml:space="preserve">feature/CS-27-ekyc</t>
+        </is>
+      </c>
+      <c r="R9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-27</t>
+        </is>
+      </c>
       <c r="S9" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">TL-06.</t>
@@ -1634,10 +1666,14 @@
       </c>
       <c r="Q10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">du-lieu-demo</t>
-        </is>
-      </c>
-      <c r="R10" s="2"/>
+          <t xml:space="preserve">feature/CS-28-du-lieu-demo</t>
+        </is>
+      </c>
+      <c r="R10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-28</t>
+        </is>
+      </c>
       <c r="S10" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Ai cần thêm dữ liệu mẫu thì nhắn Thiện hoặc tự thêm vào seeder (PR riêng).</t>
@@ -1721,10 +1757,14 @@
       </c>
       <c r="Q11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">danh-so-hop</t>
-        </is>
-      </c>
-      <c r="R11" s="2"/>
+          <t xml:space="preserve">feature/CS-29-danh-so-hop</t>
+        </is>
+      </c>
+      <c r="R11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-29</t>
+        </is>
+      </c>
       <c r="S11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Quyết định nhóm: đánh số hộp, không vẽ sơ đồ trại.</t>
@@ -1808,10 +1848,14 @@
       </c>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">cua-hang</t>
-        </is>
-      </c>
-      <c r="R12" s="2"/>
+          <t xml:space="preserve">feature/CS-30-cua-hang</t>
+        </is>
+      </c>
+      <c r="R12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-30</t>
+        </is>
+      </c>
       <c r="S12" s="2"/>
     </row>
     <row r="13">
@@ -1891,10 +1935,14 @@
       </c>
       <c r="Q13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">tai-khoan-nhan-tien</t>
-        </is>
-      </c>
-      <c r="R13" s="2"/>
+          <t xml:space="preserve">feature/CS-31-tai-khoan-nhan-tien</t>
+        </is>
+      </c>
+      <c r="R13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-31</t>
+        </is>
+      </c>
       <c r="S13" s="2"/>
     </row>
     <row r="14">
@@ -1974,10 +2022,14 @@
       </c>
       <c r="Q14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">gop-von-giu-cho</t>
-        </is>
-      </c>
-      <c r="R14" s="2"/>
+          <t xml:space="preserve">feature/CS-32-gop-von-giu-cho</t>
+        </is>
+      </c>
+      <c r="R14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-32</t>
+        </is>
+      </c>
       <c r="S14" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Luồng góp vốn tổng cộng ≤ 5 màn (Phiếu, Usability).</t>
@@ -2061,10 +2113,14 @@
       </c>
       <c r="Q15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">tao-lo-chi-phi-chuan</t>
-        </is>
-      </c>
-      <c r="R15" s="2"/>
+          <t xml:space="preserve">feature/CS-33-tao-lo-chi-phi-chuan</t>
+        </is>
+      </c>
+      <c r="R15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-33</t>
+        </is>
+      </c>
       <c r="S15" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Không có trường lợi suất kỳ vọng (BR-49).</t>
@@ -2148,10 +2204,14 @@
       </c>
       <c r="Q16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">kiem-duyet-niem-yet</t>
-        </is>
-      </c>
-      <c r="R16" s="2"/>
+          <t xml:space="preserve">feature/CS-34-kiem-duyet-niem-yet</t>
+        </is>
+      </c>
+      <c r="R16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-34</t>
+        </is>
+      </c>
       <c r="S16" s="2"/>
     </row>
     <row r="17">
@@ -2231,10 +2291,14 @@
       </c>
       <c r="Q17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ngoai-le-kyc-nguoi-dung</t>
-        </is>
-      </c>
-      <c r="R17" s="2"/>
+          <t xml:space="preserve">feature/CS-35-ngoai-le-kyc-nguoi-dung</t>
+        </is>
+      </c>
+      <c r="R17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-35</t>
+        </is>
+      </c>
       <c r="S17" s="2"/>
     </row>
     <row r="18">
@@ -2314,10 +2378,14 @@
       </c>
       <c r="Q18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">dat-hang-giu-ton</t>
-        </is>
-      </c>
-      <c r="R18" s="2"/>
+          <t xml:space="preserve">feature/CS-36-dat-hang-giu-ton</t>
+        </is>
+      </c>
+      <c r="R18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-36</t>
+        </is>
+      </c>
       <c r="S18" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">TL-28, TL-29. NFR Integrity.</t>
@@ -2401,10 +2469,14 @@
       </c>
       <c r="Q19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">canh-bao-loi</t>
-        </is>
-      </c>
-      <c r="R19" s="2"/>
+          <t xml:space="preserve">feature/CS-37-canh-bao-loi</t>
+        </is>
+      </c>
+      <c r="R19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-37</t>
+        </is>
+      </c>
       <c r="S19" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">TL-22.</t>
@@ -2488,10 +2560,14 @@
       </c>
       <c r="Q20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">thanh-toan-vietqr</t>
-        </is>
-      </c>
-      <c r="R20" s="2"/>
+          <t xml:space="preserve">feature/CS-38-thanh-toan-vietqr</t>
+        </is>
+      </c>
+      <c r="R20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-38</t>
+        </is>
+      </c>
       <c r="S20" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Báo Nhân ngay khi merge để NH-06 dùng.</t>
@@ -2575,10 +2651,14 @@
       </c>
       <c r="Q21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">duyet-lo</t>
-        </is>
-      </c>
-      <c r="R21" s="2"/>
+          <t xml:space="preserve">feature/CS-39-duyet-lo</t>
+        </is>
+      </c>
+      <c r="R21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-39</t>
+        </is>
+      </c>
       <c r="S21" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">TL-11.</t>
@@ -2662,10 +2742,14 @@
       </c>
       <c r="Q22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">canh-bao-leo-thang</t>
-        </is>
-      </c>
-      <c r="R22" s="2"/>
+          <t xml:space="preserve">feature/CS-40-canh-bao-leo-thang</t>
+        </is>
+      </c>
+      <c r="R22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-40</t>
+        </is>
+      </c>
       <c r="S22" s="2"/>
     </row>
     <row r="23">
@@ -2745,10 +2829,14 @@
       </c>
       <c r="Q23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">webhook-thanh-toan</t>
-        </is>
-      </c>
-      <c r="R23" s="2"/>
+          <t xml:space="preserve">feature/CS-41-webhook-thanh-toan</t>
+        </is>
+      </c>
+      <c r="R23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-41</t>
+        </is>
+      </c>
       <c r="S23" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">NFR Integrity: mỗi giao dịch ngân hàng ghi đúng một lần.</t>
@@ -2832,10 +2920,14 @@
       </c>
       <c r="Q24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">kham-pha-lo</t>
-        </is>
-      </c>
-      <c r="R24" s="2"/>
+          <t xml:space="preserve">feature/CS-42-kham-pha-lo</t>
+        </is>
+      </c>
+      <c r="R24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-42</t>
+        </is>
+      </c>
       <c r="S24" s="2"/>
     </row>
     <row r="25">
@@ -2915,10 +3007,14 @@
       </c>
       <c r="Q25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">gio-hang-thanh-toan</t>
-        </is>
-      </c>
-      <c r="R25" s="2"/>
+          <t xml:space="preserve">feature/CS-43-gio-hang-thanh-toan</t>
+        </is>
+      </c>
+      <c r="R25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-43</t>
+        </is>
+      </c>
       <c r="S25" s="2"/>
     </row>
     <row r="26">
@@ -2998,10 +3094,14 @@
       </c>
       <c r="Q26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">upload-bang-chung</t>
-        </is>
-      </c>
-      <c r="R26" s="2"/>
+          <t xml:space="preserve">feature/CS-44-upload-bang-chung</t>
+        </is>
+      </c>
+      <c r="R26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-44</t>
+        </is>
+      </c>
       <c r="S26" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">TL-04.</t>
@@ -3085,10 +3185,14 @@
       </c>
       <c r="Q27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">tha-giong-gan-hop</t>
-        </is>
-      </c>
-      <c r="R27" s="2"/>
+          <t xml:space="preserve">feature/CS-45-tha-giong-gan-hop</t>
+        </is>
+      </c>
+      <c r="R27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-45</t>
+        </is>
+      </c>
       <c r="S27" s="2"/>
     </row>
     <row r="28">
@@ -3168,10 +3272,14 @@
       </c>
       <c r="Q28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">theo-doi-don</t>
-        </is>
-      </c>
-      <c r="R28" s="2"/>
+          <t xml:space="preserve">feature/CS-46-theo-doi-don</t>
+        </is>
+      </c>
+      <c r="R28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-46</t>
+        </is>
+      </c>
       <c r="S28" s="2"/>
     </row>
     <row r="29">
@@ -3251,10 +3359,14 @@
       </c>
       <c r="Q29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">chot-von-hoan-tien</t>
-        </is>
-      </c>
-      <c r="R29" s="2"/>
+          <t xml:space="preserve">feature/CS-47-chot-von-hoan-tien</t>
+        </is>
+      </c>
+      <c r="R29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-47</t>
+        </is>
+      </c>
       <c r="S29" s="2"/>
     </row>
     <row r="30">
@@ -3334,10 +3446,14 @@
       </c>
       <c r="Q30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">nhat-ky-ngay</t>
-        </is>
-      </c>
-      <c r="R30" s="2"/>
+          <t xml:space="preserve">feature/CS-48-nhat-ky-ngay</t>
+        </is>
+      </c>
+      <c r="R30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-48</t>
+        </is>
+      </c>
       <c r="S30" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Hệ thống không có hệ thống nước — người nuôi tự nhập số đo.</t>
@@ -3421,10 +3537,14 @@
       </c>
       <c r="Q31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">tsk13-huan-luyen</t>
-        </is>
-      </c>
-      <c r="R31" s="2"/>
+          <t xml:space="preserve">feature/CS-49-tsk13-huan-luyen</t>
+        </is>
+      </c>
+      <c r="R31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-49</t>
+        </is>
+      </c>
       <c r="S31" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Mục tiêu precision ≥ 0,85, recall ≥ 0,80.</t>
@@ -3508,10 +3628,14 @@
       </c>
       <c r="Q32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">yeu-cau-chup-ngau-nhien</t>
-        </is>
-      </c>
-      <c r="R32" s="2"/>
+          <t xml:space="preserve">feature/CS-50-yeu-cau-chup-ngau-nhien</t>
+        </is>
+      </c>
+      <c r="R32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-50</t>
+        </is>
+      </c>
       <c r="S32" s="2"/>
     </row>
     <row r="33">
@@ -3591,10 +3715,14 @@
       </c>
       <c r="Q33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">hop-dong-ky-so</t>
-        </is>
-      </c>
-      <c r="R33" s="2"/>
+          <t xml:space="preserve">feature/CS-51-hop-dong-ky-so</t>
+        </is>
+      </c>
+      <c r="R33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-51</t>
+        </is>
+      </c>
       <c r="S33" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Ghi rõ trên PDF: mẫu chưa rà soát pháp lý, chỉ dùng demo.</t>
@@ -3678,10 +3806,14 @@
       </c>
       <c r="Q34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">su-kien-hop</t>
-        </is>
-      </c>
-      <c r="R34" s="2"/>
+          <t xml:space="preserve">feature/CS-52-su-kien-hop</t>
+        </is>
+      </c>
+      <c r="R34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-52</t>
+        </is>
+      </c>
       <c r="S34" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">TL-21. Thêm màn mới vào test/pages_smoke_test.dart.</t>
@@ -3765,10 +3897,14 @@
       </c>
       <c r="Q35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">dong-goi-quet-tem</t>
-        </is>
-      </c>
-      <c r="R35" s="2"/>
+          <t xml:space="preserve">feature/CS-53-dong-goi-quet-tem</t>
+        </is>
+      </c>
+      <c r="R35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-53</t>
+        </is>
+      </c>
       <c r="S35" s="2"/>
     </row>
     <row r="36">
@@ -3848,10 +3984,14 @@
       </c>
       <c r="Q36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">tham-dinh-bang-chung</t>
-        </is>
-      </c>
-      <c r="R36" s="2"/>
+          <t xml:space="preserve">feature/CS-54-tham-dinh-bang-chung</t>
+        </is>
+      </c>
+      <c r="R36" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-54</t>
+        </is>
+      </c>
       <c r="S36" s="2"/>
     </row>
     <row r="37">
@@ -3931,10 +4071,14 @@
       </c>
       <c r="Q37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ingestion-api</t>
-        </is>
-      </c>
-      <c r="R37" s="2"/>
+          <t xml:space="preserve">feature/CS-55-ingestion-api</t>
+        </is>
+      </c>
+      <c r="R37" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-55</t>
+        </is>
+      </c>
       <c r="S37" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Ngày nộp SRS — task nhẹ để còn thời gian viết tài liệu.</t>
@@ -4018,10 +4162,14 @@
       </c>
       <c r="Q38" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">giao-hang-nhan-hang</t>
-        </is>
-      </c>
-      <c r="R38" s="2"/>
+          <t xml:space="preserve">feature/CS-56-giao-hang-nhan-hang</t>
+        </is>
+      </c>
+      <c r="R38" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-56</t>
+        </is>
+      </c>
       <c r="S38" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">TL-31.</t>
@@ -4105,10 +4253,14 @@
       </c>
       <c r="Q39" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">giai-trinh-bang-chung</t>
-        </is>
-      </c>
-      <c r="R39" s="2"/>
+          <t xml:space="preserve">feature/CS-57-giai-trinh-bang-chung</t>
+        </is>
+      </c>
+      <c r="R39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-57</t>
+        </is>
+      </c>
       <c r="S39" s="2"/>
     </row>
     <row r="40">
@@ -4188,10 +4340,14 @@
       </c>
       <c r="Q40" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">hop-dong-ky-tay</t>
-        </is>
-      </c>
-      <c r="R40" s="2"/>
+          <t xml:space="preserve">feature/CS-58-hop-dong-ky-tay</t>
+        </is>
+      </c>
+      <c r="R40" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-58</t>
+        </is>
+      </c>
       <c r="S40" s="2"/>
     </row>
     <row r="41">
@@ -4271,10 +4427,14 @@
       </c>
       <c r="Q41" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">timeline-san-xuat</t>
-        </is>
-      </c>
-      <c r="R41" s="2"/>
+          <t xml:space="preserve">feature/CS-59-timeline-san-xuat</t>
+        </is>
+      </c>
+      <c r="R41" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-59</t>
+        </is>
+      </c>
       <c r="S41" s="2"/>
     </row>
     <row r="42">
@@ -4354,10 +4514,14 @@
       </c>
       <c r="Q42" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">khieu-nai-tranh-chap</t>
-        </is>
-      </c>
-      <c r="R42" s="2"/>
+          <t xml:space="preserve">feature/CS-60-khieu-nai-tranh-chap</t>
+        </is>
+      </c>
+      <c r="R42" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-60</t>
+        </is>
+      </c>
       <c r="S42" s="2"/>
     </row>
     <row r="43">
@@ -4437,10 +4601,14 @@
       </c>
       <c r="Q43" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">danh-muc-ndt</t>
-        </is>
-      </c>
-      <c r="R43" s="2"/>
+          <t xml:space="preserve">feature/CS-61-danh-muc-ndt</t>
+        </is>
+      </c>
+      <c r="R43" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-61</t>
+        </is>
+      </c>
       <c r="S43" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">BR-49.</t>
@@ -4524,10 +4692,14 @@
       </c>
       <c r="Q44" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">giai-ngan-doi-soat</t>
-        </is>
-      </c>
-      <c r="R44" s="2"/>
+          <t xml:space="preserve">feature/CS-62-giai-ngan-doi-soat</t>
+        </is>
+      </c>
+      <c r="R44" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-62</t>
+        </is>
+      </c>
       <c r="S44" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">TL-03.</t>
@@ -4611,10 +4783,14 @@
       </c>
       <c r="Q45" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">tsk12-property-test</t>
-        </is>
-      </c>
-      <c r="R45" s="2"/>
+          <t xml:space="preserve">feature/CS-63-tsk12-property-test</t>
+        </is>
+      </c>
+      <c r="R45" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-63</t>
+        </is>
+      </c>
       <c r="S45" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Phối hợp Thiện (TH-12) để engine có đủ hàm cho quyết toán.</t>
@@ -4698,10 +4874,14 @@
       </c>
       <c r="Q46" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">danh-gia-tra-hang</t>
-        </is>
-      </c>
-      <c r="R46" s="2"/>
+          <t xml:space="preserve">feature/CS-64-danh-gia-tra-hang</t>
+        </is>
+      </c>
+      <c r="R46" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-64</t>
+        </is>
+      </c>
       <c r="S46" s="2"/>
     </row>
     <row r="47">
@@ -4781,10 +4961,14 @@
       </c>
       <c r="Q47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">thong-bao</t>
-        </is>
-      </c>
-      <c r="R47" s="2"/>
+          <t xml:space="preserve">feature/CS-65-thong-bao</t>
+        </is>
+      </c>
+      <c r="R47" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-65</t>
+        </is>
+      </c>
       <c r="S47" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Đẩy thông báo (FCM) là phần thêm nếu còn thời gian.</t>
@@ -4868,10 +5052,14 @@
       </c>
       <c r="Q48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">cau-hinh-phi</t>
-        </is>
-      </c>
-      <c r="R48" s="2"/>
+          <t xml:space="preserve">feature/CS-66-cau-hinh-phi</t>
+        </is>
+      </c>
+      <c r="R48" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-66</t>
+        </is>
+      </c>
       <c r="S48" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Mốc M2.</t>
@@ -4955,10 +5143,14 @@
       </c>
       <c r="Q49" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">tsk12-mutation-test</t>
-        </is>
-      </c>
-      <c r="R49" s="2"/>
+          <t xml:space="preserve">feature/CS-67-tsk12-mutation-test</t>
+        </is>
+      </c>
+      <c r="R49" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-67</t>
+        </is>
+      </c>
       <c r="S49" s="2"/>
     </row>
     <row r="50">
@@ -5038,10 +5230,14 @@
       </c>
       <c r="Q50" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">dat-truoc-coc</t>
-        </is>
-      </c>
-      <c r="R50" s="2"/>
+          <t xml:space="preserve">feature/CS-68-dat-truoc-coc</t>
+        </is>
+      </c>
+      <c r="R50" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-68</t>
+        </is>
+      </c>
       <c r="S50" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Mốc M2.</t>
@@ -5125,10 +5321,14 @@
       </c>
       <c r="Q51" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">hoan-thien-mobile</t>
-        </is>
-      </c>
-      <c r="R51" s="2"/>
+          <t xml:space="preserve">feature/CS-69-hoan-thien-mobile</t>
+        </is>
+      </c>
+      <c r="R51" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-69</t>
+        </is>
+      </c>
       <c r="S51" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Mốc M2.</t>
@@ -5212,10 +5412,14 @@
       </c>
       <c r="Q52" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">tinh-quyet-toan</t>
-        </is>
-      </c>
-      <c r="R52" s="2"/>
+          <t xml:space="preserve">feature/CS-70-tinh-quyet-toan</t>
+        </is>
+      </c>
+      <c r="R52" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-70</t>
+        </is>
+      </c>
       <c r="S52" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Phối hợp Viên (TSK-12) dùng chung bộ test.</t>
@@ -5299,10 +5503,14 @@
       </c>
       <c r="Q53" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">thu-hoach-can-hang</t>
-        </is>
-      </c>
-      <c r="R53" s="2"/>
+          <t xml:space="preserve">feature/CS-71-thu-hoach-can-hang</t>
+        </is>
+      </c>
+      <c r="R53" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-71</t>
+        </is>
+      </c>
       <c r="S53" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Mở cửa sổ bao tiêu cho NH-15.</t>
@@ -5386,10 +5594,14 @@
       </c>
       <c r="Q54" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">cam-ket-bao-tieu</t>
-        </is>
-      </c>
-      <c r="R54" s="2"/>
+          <t xml:space="preserve">feature/CS-72-cam-ket-bao-tieu</t>
+        </is>
+      </c>
+      <c r="R54" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-72</t>
+        </is>
+      </c>
       <c r="S54" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">TL-30.</t>
@@ -5473,10 +5685,14 @@
       </c>
       <c r="Q55" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">dashboard</t>
-        </is>
-      </c>
-      <c r="R55" s="2"/>
+          <t xml:space="preserve">feature/CS-73-dashboard</t>
+        </is>
+      </c>
+      <c r="R55" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-73</t>
+        </is>
+      </c>
       <c r="S55" s="2"/>
     </row>
     <row r="56">
@@ -5556,10 +5772,14 @@
       </c>
       <c r="Q56" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">in-kich-hoat-tem</t>
-        </is>
-      </c>
-      <c r="R56" s="2"/>
+          <t xml:space="preserve">feature/CS-74-in-kich-hoat-tem</t>
+        </is>
+      </c>
+      <c r="R56" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-74</t>
+        </is>
+      </c>
       <c r="S56" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Máy in nhãn là phần cứng ngoài phạm vi — chỉ xuất nội dung in.</t>
@@ -5643,10 +5863,14 @@
       </c>
       <c r="Q57" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">nhan-hang-bao-tieu</t>
-        </is>
-      </c>
-      <c r="R57" s="2"/>
+          <t xml:space="preserve">feature/CS-75-nhan-hang-bao-tieu</t>
+        </is>
+      </c>
+      <c r="R57" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-75</t>
+        </is>
+      </c>
       <c r="S57" s="2"/>
     </row>
     <row r="58">
@@ -5726,10 +5950,14 @@
       </c>
       <c r="Q58" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">xuat-nhat-ky-kiem-toan</t>
-        </is>
-      </c>
-      <c r="R58" s="2"/>
+          <t xml:space="preserve">feature/CS-76-xuat-nhat-ky-kiem-toan</t>
+        </is>
+      </c>
+      <c r="R58" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-76</t>
+        </is>
+      </c>
       <c r="S58" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">TL-08.</t>
@@ -5813,10 +6041,14 @@
       </c>
       <c r="Q59" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">cong-bo-sao-ke-gop-y</t>
-        </is>
-      </c>
-      <c r="R59" s="2"/>
+          <t xml:space="preserve">feature/CS-77-cong-bo-sao-ke-gop-y</t>
+        </is>
+      </c>
+      <c r="R59" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-77</t>
+        </is>
+      </c>
       <c r="S59" s="2"/>
     </row>
     <row r="60">
@@ -5896,10 +6128,14 @@
       </c>
       <c r="Q60" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">chot-thu-hoach-ton-kho</t>
-        </is>
-      </c>
-      <c r="R60" s="2"/>
+          <t xml:space="preserve">feature/CS-78-chot-thu-hoach-ton-kho</t>
+        </is>
+      </c>
+      <c r="R60" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-78</t>
+        </is>
+      </c>
       <c r="S60" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">TL-23.</t>
@@ -5983,10 +6219,14 @@
       </c>
       <c r="Q61" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">tsk13-tich-hop</t>
-        </is>
-      </c>
-      <c r="R61" s="2"/>
+          <t xml:space="preserve">feature/CS-79-tsk13-tich-hop</t>
+        </is>
+      </c>
+      <c r="R61" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-79</t>
+        </is>
+      </c>
       <c r="S61" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">File .onnx đưa lên GitHub Releases, không commit.</t>
@@ -6070,10 +6310,14 @@
       </c>
       <c r="Q62" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">trien-khai-server</t>
-        </is>
-      </c>
-      <c r="R62" s="2"/>
+          <t xml:space="preserve">feature/CS-80-trien-khai-server</t>
+        </is>
+      </c>
+      <c r="R62" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-80</t>
+        </is>
+      </c>
       <c r="S62" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Mốc M3.</t>
@@ -6157,10 +6401,14 @@
       </c>
       <c r="Q63" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">duyet-chi-tra</t>
-        </is>
-      </c>
-      <c r="R63" s="2"/>
+          <t xml:space="preserve">feature/CS-81-duyet-chi-tra</t>
+        </is>
+      </c>
+      <c r="R63" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-81</t>
+        </is>
+      </c>
       <c r="S63" s="2"/>
     </row>
     <row r="64">
@@ -6240,10 +6488,14 @@
       </c>
       <c r="Q64" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">truy-xuat-tem</t>
-        </is>
-      </c>
-      <c r="R64" s="2"/>
+          <t xml:space="preserve">feature/CS-82-truy-xuat-tem</t>
+        </is>
+      </c>
+      <c r="R64" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-82</t>
+        </is>
+      </c>
       <c r="S64" s="2"/>
     </row>
     <row r="65">
@@ -6323,10 +6575,14 @@
       </c>
       <c r="Q65" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ke-hoach-kiem-thu</t>
-        </is>
-      </c>
-      <c r="R65" s="2"/>
+          <t xml:space="preserve">feature/CS-83-ke-hoach-kiem-thu</t>
+        </is>
+      </c>
+      <c r="R65" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-83</t>
+        </is>
+      </c>
       <c r="S65" s="2"/>
     </row>
     <row r="66">
@@ -6406,10 +6662,14 @@
       </c>
       <c r="Q66" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">phat-hanh-app</t>
-        </is>
-      </c>
-      <c r="R66" s="2"/>
+          <t xml:space="preserve">feature/CS-84-phat-hanh-app</t>
+        </is>
+      </c>
+      <c r="R66" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-84</t>
+        </is>
+      </c>
       <c r="S66" s="2"/>
     </row>
     <row r="67">
@@ -6489,10 +6749,14 @@
       </c>
       <c r="Q67" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ra-soat-duong-tien</t>
-        </is>
-      </c>
-      <c r="R67" s="2"/>
+          <t xml:space="preserve">feature/CS-85-ra-soat-duong-tien</t>
+        </is>
+      </c>
+      <c r="R67" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-85</t>
+        </is>
+      </c>
       <c r="S67" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Mốc M3.</t>
@@ -6576,10 +6840,14 @@
       </c>
       <c r="Q68" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">tsk12-ket-qua</t>
-        </is>
-      </c>
-      <c r="R68" s="2"/>
+          <t xml:space="preserve">feature/CS-86-tsk12-ket-qua</t>
+        </is>
+      </c>
+      <c r="R68" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-86</t>
+        </is>
+      </c>
       <c r="S68" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Mốc M3.</t>
@@ -6663,10 +6931,14 @@
       </c>
       <c r="Q69" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">kiem-thu-tai</t>
-        </is>
-      </c>
-      <c r="R69" s="2"/>
+          <t xml:space="preserve">feature/CS-87-kiem-thu-tai</t>
+        </is>
+      </c>
+      <c r="R69" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-87</t>
+        </is>
+      </c>
       <c r="S69" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Chạy trên server thật sau khi deploy (KH-16).</t>
@@ -6750,10 +7022,14 @@
       </c>
       <c r="Q70" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">bao-mat</t>
-        </is>
-      </c>
-      <c r="R70" s="2"/>
+          <t xml:space="preserve">feature/CS-88-bao-mat</t>
+        </is>
+      </c>
+      <c r="R70" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-88</t>
+        </is>
+      </c>
       <c r="S70" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">NFR Security.</t>
@@ -6837,10 +7113,14 @@
       </c>
       <c r="Q71" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">demo-dau-cuoi</t>
-        </is>
-      </c>
-      <c r="R71" s="2"/>
+          <t xml:space="preserve">feature/CS-89-demo-dau-cuoi</t>
+        </is>
+      </c>
+      <c r="R71" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-89</t>
+        </is>
+      </c>
       <c r="S71" s="2"/>
     </row>
     <row r="72">
@@ -6920,10 +7200,14 @@
       </c>
       <c r="Q72" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">kiem-thu-san-xuat</t>
-        </is>
-      </c>
-      <c r="R72" s="2"/>
+          <t xml:space="preserve">feature/CS-90-kiem-thu-san-xuat</t>
+        </is>
+      </c>
+      <c r="R72" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-90</t>
+        </is>
+      </c>
       <c r="S72" s="2"/>
     </row>
     <row r="73">
@@ -7003,10 +7287,14 @@
       </c>
       <c r="Q73" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">chay-kiem-thu</t>
-        </is>
-      </c>
-      <c r="R73" s="2"/>
+          <t xml:space="preserve">feature/CS-91-chay-kiem-thu</t>
+        </is>
+      </c>
+      <c r="R73" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-91</t>
+        </is>
+      </c>
       <c r="S73" s="2"/>
     </row>
     <row r="74">
@@ -7086,10 +7374,14 @@
       </c>
       <c r="Q74" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">kiem-thu-mobile</t>
-        </is>
-      </c>
-      <c r="R74" s="2"/>
+          <t xml:space="preserve">feature/CS-92-kiem-thu-mobile</t>
+        </is>
+      </c>
+      <c r="R74" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-92</t>
+        </is>
+      </c>
       <c r="S74" s="2"/>
     </row>
     <row r="75">
@@ -7169,10 +7461,14 @@
       </c>
       <c r="Q75" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">chot-ban-demo</t>
-        </is>
-      </c>
-      <c r="R75" s="2"/>
+          <t xml:space="preserve">feature/CS-93-chot-ban-demo</t>
+        </is>
+      </c>
+      <c r="R75" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CS-93</t>
+        </is>
+      </c>
       <c r="S75" s="2"/>
     </row>
   </sheetData>
@@ -7276,23 +7572,23 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TH-01 Khởi động: cả nhóm chạy được dự án, bảo vệ nhánh main/develop, dựng board Jira
-TH-02 Nhật ký kiểm toán dùng chung + khung job nền (ngày 1/2)</t>
+          <t xml:space="preserve">CS-20 · TH-01 Khởi động: cả nhóm chạy được dự án, bảo vệ nhánh main/develop, dựng board Jira
+CS-21 · TH-02 Nhật ký kiểm toán dùng chung + khung job nền (ngày 1/2)</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">VI-01 Đăng ký hồ sơ hộ nuôi</t>
+          <t xml:space="preserve">CS-22 · VI-01 Đăng ký hồ sơ hộ nuôi</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NH-01 TSK-13: kế hoạch dữ liệu ảnh + bắt đầu gán nhãn</t>
+          <t xml:space="preserve">CS-23 · NH-01 TSK-13: kế hoạch dữ liệu ảnh + bắt đầu gán nhãn</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">KH-01 Mobile chạy trên Android + thêm package cho các task sau</t>
+          <t xml:space="preserve">CS-24 · KH-01 Mobile chạy trên Android + thêm package cho các task sau</t>
         </is>
       </c>
       <c r="H2" s="9" t="inlineStr">
@@ -7317,22 +7613,22 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TH-02 Nhật ký kiểm toán dùng chung + khung job nền (ngày 2/2)</t>
+          <t xml:space="preserve">CS-21 · TH-02 Nhật ký kiểm toán dùng chung + khung job nền (ngày 2/2)</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">VI-02 Duyệt hộ nuôi + quản lý nhân viên hộ nuôi</t>
+          <t xml:space="preserve">CS-25 · VI-02 Duyệt hộ nuôi + quản lý nhân viên hộ nuôi</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NH-02 Niêm yết sản phẩm</t>
+          <t xml:space="preserve">CS-26 · NH-02 Niêm yết sản phẩm</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">KH-02 Xác minh danh tính (eKYC) — mobile + web</t>
+          <t xml:space="preserve">CS-27 · KH-02 Xác minh danh tính (eKYC) — mobile + web</t>
         </is>
       </c>
       <c r="H3" s="2"/>
@@ -7353,22 +7649,22 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TH-03 Dữ liệu demo đủ vòng đời để cả nhóm làm song song</t>
+          <t xml:space="preserve">CS-28 · TH-03 Dữ liệu demo đủ vòng đời để cả nhóm làm song song</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">VI-03 Đánh số hộp nuôi (thay sơ đồ trại)</t>
+          <t xml:space="preserve">CS-29 · VI-03 Đánh số hộp nuôi (thay sơ đồ trại)</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NH-03 Cửa hàng: duyệt, lọc, sắp xếp sản phẩm</t>
+          <t xml:space="preserve">CS-30 · NH-03 Cửa hàng: duyệt, lọc, sắp xếp sản phẩm</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">KH-03 Tài khoản nhận tiền + sổ địa chỉ giao hàng</t>
+          <t xml:space="preserve">CS-31 · KH-03 Tài khoản nhận tiền + sổ địa chỉ giao hàng</t>
         </is>
       </c>
       <c r="H4" s="2"/>
@@ -7389,22 +7685,22 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TH-04 Xác nhận rủi ro + giữ chỗ góp vốn (luồng góp vốn màn 1–2) (ngày 1/2)</t>
+          <t xml:space="preserve">CS-32 · TH-04 Xác nhận rủi ro + giữ chỗ góp vốn (luồng góp vốn màn 1–2) (ngày 1/2)</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">VI-04 Tạo lô + soạn chi phí chuẩn (ngày 1/2)</t>
+          <t xml:space="preserve">CS-33 · VI-04 Tạo lô + soạn chi phí chuẩn (ngày 1/2)</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NH-04 Kiểm duyệt niêm yết + cảnh báo sắp hết hàng</t>
+          <t xml:space="preserve">CS-34 · NH-04 Kiểm duyệt niêm yết + cảnh báo sắp hết hàng</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">KH-04 Ngoại lệ KYC + quản lý người dùng</t>
+          <t xml:space="preserve">CS-35 · KH-04 Ngoại lệ KYC + quản lý người dùng</t>
         </is>
       </c>
       <c r="H5" s="2"/>
@@ -7425,22 +7721,22 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TH-04 Xác nhận rủi ro + giữ chỗ góp vốn (luồng góp vốn màn 1–2) (ngày 2/2)</t>
+          <t xml:space="preserve">CS-32 · TH-04 Xác nhận rủi ro + giữ chỗ góp vốn (luồng góp vốn màn 1–2) (ngày 2/2)</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">VI-04 Tạo lô + soạn chi phí chuẩn (ngày 2/2)</t>
+          <t xml:space="preserve">CS-33 · VI-04 Tạo lô + soạn chi phí chuẩn (ngày 2/2)</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NH-05 Đặt hàng: giữ tồn nguyên tử, không bán vượt (ngày 1/2)</t>
+          <t xml:space="preserve">CS-36 · NH-05 Đặt hàng: giữ tồn nguyên tử, không bán vượt (ngày 1/2)</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">KH-05 Cảnh báo — lõi dùng chung + xác nhận cảnh báo</t>
+          <t xml:space="preserve">CS-37 · KH-05 Cảnh báo — lõi dùng chung + xác nhận cảnh báo</t>
         </is>
       </c>
       <c r="H6" s="2"/>
@@ -7461,22 +7757,22 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TH-05 Thanh toán VietQR (dùng chung cho góp vốn, đơn hàng, cọc)</t>
+          <t xml:space="preserve">CS-38 · TH-05 Thanh toán VietQR (dùng chung cho góp vốn, đơn hàng, cọc)</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">VI-05 Duyệt lô: mở gọi vốn + khoá chi phí chuẩn</t>
+          <t xml:space="preserve">CS-39 · VI-05 Duyệt lô: mở gọi vốn + khoá chi phí chuẩn</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NH-05 Đặt hàng: giữ tồn nguyên tử, không bán vượt (ngày 2/2)</t>
+          <t xml:space="preserve">CS-36 · NH-05 Đặt hàng: giữ tồn nguyên tử, không bán vượt (ngày 2/2)</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">KH-06 Cảnh báo — job leo thang + màn quản trị</t>
+          <t xml:space="preserve">CS-40 · KH-06 Cảnh báo — job leo thang + màn quản trị</t>
         </is>
       </c>
       <c r="H7" s="2"/>
@@ -7497,22 +7793,22 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TH-06 Webhook thanh toán (chống trùng) + giả lập chuyển khoản (ngày 1/2)</t>
+          <t xml:space="preserve">CS-41 · TH-06 Webhook thanh toán (chống trùng) + giả lập chuyển khoản (ngày 1/2)</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">VI-06 Khám phá lô (web + mobile)</t>
+          <t xml:space="preserve">CS-42 · VI-06 Khám phá lô (web + mobile)</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NH-06 Giỏ hàng + thanh toán trên web</t>
+          <t xml:space="preserve">CS-43 · NH-06 Giỏ hàng + thanh toán trên web</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">KH-07 Chụp &amp; gửi bằng chứng (mobile) + xử lý ảnh trên server (ngày 1/2)</t>
+          <t xml:space="preserve">CS-44 · KH-07 Chụp &amp; gửi bằng chứng (mobile) + xử lý ảnh trên server (ngày 1/2)</t>
         </is>
       </c>
       <c r="H8" s="9" t="inlineStr">
@@ -7537,22 +7833,22 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TH-06 Webhook thanh toán (chống trùng) + giả lập chuyển khoản (ngày 2/2)</t>
+          <t xml:space="preserve">CS-41 · TH-06 Webhook thanh toán (chống trùng) + giả lập chuyển khoản (ngày 2/2)</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">VI-07 Thả giống: gán hộp cho lô, tạo từng con cua</t>
+          <t xml:space="preserve">CS-45 · VI-07 Thả giống: gán hộp cho lô, tạo từng con cua</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NH-07 Theo dõi đơn, lịch sử, huỷ + job trả tồn quá hạn</t>
+          <t xml:space="preserve">CS-46 · NH-07 Theo dõi đơn, lịch sử, huỷ + job trả tồn quá hạn</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">KH-07 Chụp &amp; gửi bằng chứng (mobile) + xử lý ảnh trên server (ngày 2/2)</t>
+          <t xml:space="preserve">CS-44 · KH-07 Chụp &amp; gửi bằng chứng (mobile) + xử lý ảnh trên server (ngày 2/2)</t>
         </is>
       </c>
       <c r="H9" s="2"/>
@@ -7573,22 +7869,22 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TH-07 Job hết hạn giữ chỗ, chốt vốn hoặc huỷ lô + hoàn tiền</t>
+          <t xml:space="preserve">CS-47 · TH-07 Job hết hạn giữ chỗ, chốt vốn hoặc huỷ lô + hoàn tiền</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">VI-08 Nhật ký ngày (pH, nhiệt độ nước, độ mặn, thức ăn) — web + mobile</t>
+          <t xml:space="preserve">CS-48 · VI-08 Nhật ký ngày (pH, nhiệt độ nước, độ mặn, thức ăn) — web + mobile</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NH-08 TSK-13: huấn luyện mô hình lần 1 + đánh giá</t>
+          <t xml:space="preserve">CS-49 · NH-08 TSK-13: huấn luyện mô hình lần 1 + đánh giá</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">KH-08 Yêu cầu chụp ngẫu nhiên</t>
+          <t xml:space="preserve">CS-50 · KH-08 Yêu cầu chụp ngẫu nhiên</t>
         </is>
       </c>
       <c r="H10" s="2"/>
@@ -7609,22 +7905,22 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TH-08 Hợp đồng: sinh từ mẫu + ký số theo thứ tự (Operator → Investor) (ngày 1/2)</t>
+          <t xml:space="preserve">CS-51 · TH-08 Hợp đồng: sinh từ mẫu + ký số theo thứ tự (Operator → Investor) (ngày 1/2)</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">VI-09 Sự kiện từng hộp: lột xác, chết, thả bù, chuyển hộp</t>
+          <t xml:space="preserve">CS-52 · VI-09 Sự kiện từng hộp: lột xác, chết, thả bù, chuyển hộp</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NH-09 Đóng gói đơn bằng quét tem (mobile hộ nuôi)</t>
+          <t xml:space="preserve">CS-53 · NH-09 Đóng gói đơn bằng quét tem (mobile hộ nuôi)</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">KH-09 Thẩm định bằng chứng bị gắn cờ</t>
+          <t xml:space="preserve">CS-54 · KH-09 Thẩm định bằng chứng bị gắn cờ</t>
         </is>
       </c>
       <c r="H11" s="2"/>
@@ -7645,22 +7941,22 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TH-08 Hợp đồng: sinh từ mẫu + ký số theo thứ tự (Operator → Investor) (ngày 2/2)</t>
+          <t xml:space="preserve">CS-51 · TH-08 Hợp đồng: sinh từ mẫu + ký số theo thứ tự (Operator → Investor) (ngày 2/2)</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">VI-10 Ingestion API cho phần mềm của trại + đặc tả</t>
+          <t xml:space="preserve">CS-55 · VI-10 Ingestion API cho phần mềm của trại + đặc tả</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NH-10 Giao hàng + xác nhận đã nhận → hoàn tất đơn</t>
+          <t xml:space="preserve">CS-56 · NH-10 Giao hàng + xác nhận đã nhận → hoàn tất đơn</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">KH-10 Giải trình bằng chứng</t>
+          <t xml:space="preserve">CS-57 · KH-10 Giải trình bằng chứng</t>
         </is>
       </c>
       <c r="H12" s="9" t="inlineStr">
@@ -7685,22 +7981,22 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TH-09 Hợp đồng ký tay (tải bản scan) + kho hợp đồng</t>
+          <t xml:space="preserve">CS-58 · TH-09 Hợp đồng ký tay (tải bản scan) + kho hợp đồng</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">VI-11 Timeline sản xuất cho nhà đầu tư</t>
+          <t xml:space="preserve">CS-59 · VI-11 Timeline sản xuất cho nhà đầu tư</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NH-11 Khiếu nại + giải quyết tranh chấp</t>
+          <t xml:space="preserve">CS-60 · NH-11 Khiếu nại + giải quyết tranh chấp</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">KH-11 Danh mục nhà đầu tư — mobile + web</t>
+          <t xml:space="preserve">CS-61 · KH-11 Danh mục nhà đầu tư — mobile + web</t>
         </is>
       </c>
       <c r="H13" s="2"/>
@@ -7721,22 +8017,22 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TH-10 Giải ngân theo mốc + đối soát chi trả</t>
+          <t xml:space="preserve">CS-62 · TH-10 Giải ngân theo mốc + đối soát chi trả</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">VI-12 TSK-12: property-based + metamorphic + model-based test cho engine quyết toán</t>
+          <t xml:space="preserve">CS-63 · VI-12 TSK-12: property-based + metamorphic + model-based test cho engine quyết toán</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NH-12 Đánh giá đơn hàng + trả hàng</t>
+          <t xml:space="preserve">CS-64 · NH-12 Đánh giá đơn hàng + trả hàng</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">KH-12 Thông báo trong app</t>
+          <t xml:space="preserve">CS-65 · KH-12 Thông báo trong app</t>
         </is>
       </c>
       <c r="H14" s="2"/>
@@ -7757,22 +8053,22 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TH-11 Cấu hình bậc phí nền tảng + tích hợp giữa kỳ</t>
+          <t xml:space="preserve">CS-66 · TH-11 Cấu hình bậc phí nền tảng + tích hợp giữa kỳ</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">VI-13 TSK-12: mutation testing bằng Stryker.NET</t>
+          <t xml:space="preserve">CS-67 · VI-13 TSK-12: mutation testing bằng Stryker.NET</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NH-13 Đặt trước có cọc cho lô đang nuôi</t>
+          <t xml:space="preserve">CS-68 · NH-13 Đặt trước có cọc cho lô đang nuôi</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">KH-13 Hoàn thiện mobile giữa kỳ</t>
+          <t xml:space="preserve">CS-69 · KH-13 Hoàn thiện mobile giữa kỳ</t>
         </is>
       </c>
       <c r="H15" s="9" t="inlineStr">
@@ -7797,22 +8093,22 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TH-12 Tính quyết toán (Revenue Pool, thù lao, chia theo vốn, thuế) (ngày 1/2)</t>
+          <t xml:space="preserve">CS-70 · TH-12 Tính quyết toán (Revenue Pool, thù lao, chia theo vốn, thuế) (ngày 1/2)</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">VI-14 Thu hoạch: cân từng con, xếp hạng, tạo tem</t>
+          <t xml:space="preserve">CS-71 · VI-14 Thu hoạch: cân từng con, xếp hạng, tạo tem</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NH-14 Cam kết bao tiêu</t>
+          <t xml:space="preserve">CS-72 · NH-14 Cam kết bao tiêu</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">KH-14 Dashboard quản trị + hộ nuôi</t>
+          <t xml:space="preserve">CS-73 · KH-14 Dashboard quản trị + hộ nuôi</t>
         </is>
       </c>
       <c r="H16" s="2"/>
@@ -7833,22 +8129,22 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TH-12 Tính quyết toán (Revenue Pool, thù lao, chia theo vốn, thuế) (ngày 2/2)</t>
+          <t xml:space="preserve">CS-70 · TH-12 Tính quyết toán (Revenue Pool, thù lao, chia theo vốn, thuế) (ngày 2/2)</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">VI-15 In tem + kích hoạt tem bằng ảnh xác nhận</t>
+          <t xml:space="preserve">CS-74 · VI-15 In tem + kích hoạt tem bằng ảnh xác nhận</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NH-15 Nhận hàng bao tiêu trong cửa sổ ưu tiên</t>
+          <t xml:space="preserve">CS-75 · NH-15 Nhận hàng bao tiêu trong cửa sổ ưu tiên</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">KH-15 Xem + xuất nhật ký kiểm toán</t>
+          <t xml:space="preserve">CS-76 · KH-15 Xem + xuất nhật ký kiểm toán</t>
         </is>
       </c>
       <c r="H17" s="2"/>
@@ -7869,22 +8165,22 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TH-13 Công bố quyết toán + sao kê NĐT + góp ý trong hạn</t>
+          <t xml:space="preserve">CS-77 · TH-13 Công bố quyết toán + sao kê NĐT + góp ý trong hạn</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">VI-16 Chốt đợt thu hoạch → tồn kho cho cửa hàng</t>
+          <t xml:space="preserve">CS-78 · VI-16 Chốt đợt thu hoạch → tồn kho cho cửa hàng</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NH-16 TSK-13: xuất ONNX + tích hợp vào API</t>
+          <t xml:space="preserve">CS-79 · NH-16 TSK-13: xuất ONNX + tích hợp vào API</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">KH-16 Triển khai lên server</t>
+          <t xml:space="preserve">CS-80 · KH-16 Triển khai lên server</t>
         </is>
       </c>
       <c r="H18" s="2"/>
@@ -7905,22 +8201,22 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TH-14 Duyệt quyết toán + phát lệnh chi trả + đóng lô</t>
+          <t xml:space="preserve">CS-81 · TH-14 Duyệt quyết toán + phát lệnh chi trả + đóng lô</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">VI-17 Truy xuất bằng tem (công khai) — web + mobile</t>
+          <t xml:space="preserve">CS-82 · VI-17 Truy xuất bằng tem (công khai) — web + mobile</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NH-17 Kế hoạch + ca kiểm thử hệ thống</t>
+          <t xml:space="preserve">CS-83 · NH-17 Kế hoạch + ca kiểm thử hệ thống</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">KH-17 Phát hành app cho demo</t>
+          <t xml:space="preserve">CS-84 · KH-17 Phát hành app cho demo</t>
         </is>
       </c>
       <c r="H19" s="2"/>
@@ -7941,22 +8237,22 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TH-15 Rà soát mọi đường tiền + nhật ký kiểm toán</t>
+          <t xml:space="preserve">CS-85 · TH-15 Rà soát mọi đường tiền + nhật ký kiểm toán</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">VI-18 TSK-12: tổng hợp kết quả nghiên cứu + test quyết toán với dữ liệu thật</t>
+          <t xml:space="preserve">CS-86 · VI-18 TSK-12: tổng hợp kết quả nghiên cứu + test quyết toán với dữ liệu thật</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NH-18 Kiểm thử tải và đồng thời</t>
+          <t xml:space="preserve">CS-87 · NH-18 Kiểm thử tải và đồng thời</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">KH-18 Rà bảo mật + phân quyền</t>
+          <t xml:space="preserve">CS-88 · KH-18 Rà bảo mật + phân quyền</t>
         </is>
       </c>
       <c r="H20" s="9" t="inlineStr">
@@ -7981,22 +8277,22 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TH-16 Chạy kịch bản demo đầu-cuối lần 1 (cả nhóm) + sửa lỗi</t>
+          <t xml:space="preserve">CS-89 · TH-16 Chạy kịch bản demo đầu-cuối lần 1 (cả nhóm) + sửa lỗi</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">VI-19 Kiểm thử đầu-cuối nhánh hộ nuôi → sản xuất → thu hoạch + sửa lỗi (ngày 1/2)</t>
+          <t xml:space="preserve">CS-90 · VI-19 Kiểm thử đầu-cuối nhánh hộ nuôi → sản xuất → thu hoạch + sửa lỗi (ngày 1/2)</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NH-19 Chạy ca kiểm thử, báo lỗi, báo cáo kiểm thử (ngày 1/2)</t>
+          <t xml:space="preserve">CS-91 · NH-19 Chạy ca kiểm thử, báo lỗi, báo cáo kiểm thử (ngày 1/2)</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">KH-19 Kiểm thử đầu-cuối trên server + chuẩn bị máy demo (ngày 1/2)</t>
+          <t xml:space="preserve">CS-92 · KH-19 Kiểm thử đầu-cuối trên server + chuẩn bị máy demo (ngày 1/2)</t>
         </is>
       </c>
       <c r="H21" s="2"/>
@@ -8017,22 +8313,22 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TH-17 Chốt bản demo v1.0 + tập dượt</t>
+          <t xml:space="preserve">CS-93 · TH-17 Chốt bản demo v1.0 + tập dượt</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">VI-19 Kiểm thử đầu-cuối nhánh hộ nuôi → sản xuất → thu hoạch + sửa lỗi (ngày 2/2)</t>
+          <t xml:space="preserve">CS-90 · VI-19 Kiểm thử đầu-cuối nhánh hộ nuôi → sản xuất → thu hoạch + sửa lỗi (ngày 2/2)</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NH-19 Chạy ca kiểm thử, báo lỗi, báo cáo kiểm thử (ngày 2/2)</t>
+          <t xml:space="preserve">CS-91 · NH-19 Chạy ca kiểm thử, báo lỗi, báo cáo kiểm thử (ngày 2/2)</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">KH-19 Kiểm thử đầu-cuối trên server + chuẩn bị máy demo (ngày 2/2)</t>
+          <t xml:space="preserve">CS-92 · KH-19 Kiểm thử đầu-cuối trên server + chuẩn bị máy demo (ngày 2/2)</t>
         </is>
       </c>
       <c r="H22" s="9" t="inlineStr">

</xml_diff>